<commit_message>
Seguimiento de cuentas · LS · 2026-09-15 18:08
</commit_message>
<xml_diff>
--- a/data/seguimiento_cuentas.xlsx
+++ b/data/seguimiento_cuentas.xlsx
@@ -22677,7 +22677,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J163"/>
+  <dimension ref="A1:J165"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -28649,6 +28649,74 @@
       </c>
       <c r="I163" t="inlineStr"/>
       <c r="J163" t="inlineStr"/>
+    </row>
+    <row r="164">
+      <c r="A164" s="1" t="n">
+        <v>46280</v>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>Remunerada</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>Banco Supervielle</t>
+        </is>
+      </c>
+      <c r="D164" t="inlineStr">
+        <is>
+          <t>Novus PyME FCI Abierto PyMES</t>
+        </is>
+      </c>
+      <c r="E164" t="inlineStr"/>
+      <c r="F164" t="inlineStr">
+        <is>
+          <t>Abierta</t>
+        </is>
+      </c>
+      <c r="G164" t="inlineStr"/>
+      <c r="H164" t="inlineStr">
+        <is>
+          <t>4. Exención ARCA</t>
+        </is>
+      </c>
+      <c r="I164" t="inlineStr"/>
+      <c r="J164" t="inlineStr"/>
+    </row>
+    <row r="165">
+      <c r="A165" s="1" t="n">
+        <v>46280</v>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>Remunerada</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>Banco Supervielle</t>
+        </is>
+      </c>
+      <c r="D165" t="inlineStr">
+        <is>
+          <t>Novus Renta Variable</t>
+        </is>
+      </c>
+      <c r="E165" t="inlineStr"/>
+      <c r="F165" t="inlineStr">
+        <is>
+          <t>En proceso</t>
+        </is>
+      </c>
+      <c r="G165" t="inlineStr"/>
+      <c r="H165" t="inlineStr">
+        <is>
+          <t>3. Doc SD</t>
+        </is>
+      </c>
+      <c r="I165" t="inlineStr"/>
+      <c r="J165" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Seguimiento de cuentas · LS · 2026-09-16 17:41
</commit_message>
<xml_diff>
--- a/data/seguimiento_cuentas.xlsx
+++ b/data/seguimiento_cuentas.xlsx
@@ -22677,7 +22677,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J165"/>
+  <dimension ref="A1:J166"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -28717,6 +28717,40 @@
       </c>
       <c r="I165" t="inlineStr"/>
       <c r="J165" t="inlineStr"/>
+    </row>
+    <row r="166">
+      <c r="A166" s="1" t="n">
+        <v>46281</v>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>Remunerada</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>Banco Supervielle</t>
+        </is>
+      </c>
+      <c r="D166" t="inlineStr">
+        <is>
+          <t>Novus Renta Capital</t>
+        </is>
+      </c>
+      <c r="E166" t="inlineStr"/>
+      <c r="F166" t="inlineStr">
+        <is>
+          <t>Abierta</t>
+        </is>
+      </c>
+      <c r="G166" t="inlineStr"/>
+      <c r="H166" t="inlineStr">
+        <is>
+          <t>5. Habilitada para operar</t>
+        </is>
+      </c>
+      <c r="I166" t="inlineStr"/>
+      <c r="J166" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Seguimiento de cuentas · LS · 2026-09-16 18:25
</commit_message>
<xml_diff>
--- a/data/seguimiento_cuentas.xlsx
+++ b/data/seguimiento_cuentas.xlsx
@@ -23128,7 +23128,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>NOVUS MULTIESTRATEGIA</t>
+          <t>Novus Multiestrategia</t>
         </is>
       </c>
       <c r="E12" t="inlineStr"/>
@@ -23166,7 +23166,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>NOVUS RENTA FIJA</t>
+          <t>Novus Renta Fija</t>
         </is>
       </c>
       <c r="E13" t="inlineStr"/>
@@ -23204,7 +23204,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>NOVUS RENTA MIXTA FCI</t>
+          <t>Novus Renta Mixta</t>
         </is>
       </c>
       <c r="E14" t="inlineStr"/>
@@ -23242,7 +23242,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>NOVUS RENTA CAPITAL</t>
+          <t>Novus Renta Capital</t>
         </is>
       </c>
       <c r="E15" t="inlineStr"/>
@@ -23280,7 +23280,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>NOVUS GESTION FCI</t>
+          <t>Novus Gestión</t>
         </is>
       </c>
       <c r="E16" t="inlineStr"/>
@@ -23318,7 +23318,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>NOVUS RENTA BALANCEADO</t>
+          <t>Novus Renta Balanceado</t>
         </is>
       </c>
       <c r="E17" t="inlineStr"/>
@@ -23356,7 +23356,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>NOVUS LIQUIDEZ PLUS</t>
+          <t>Novus Liquidez Plus</t>
         </is>
       </c>
       <c r="E18" t="inlineStr"/>
@@ -23394,7 +23394,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>NOVUS VALOR</t>
+          <t>Novus Valor</t>
         </is>
       </c>
       <c r="E19" t="inlineStr"/>
@@ -23432,7 +23432,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>NOVUS INCOME</t>
+          <t>Novus Income</t>
         </is>
       </c>
       <c r="E20" t="inlineStr"/>
@@ -23470,7 +23470,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>NOVUS ESTRATEGIA</t>
+          <t>Novus Estrategia</t>
         </is>
       </c>
       <c r="E21" t="inlineStr"/>
@@ -23508,7 +23508,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>NOVUS GESTION II</t>
+          <t>Novus Gestion II</t>
         </is>
       </c>
       <c r="E22" t="inlineStr"/>
@@ -23546,7 +23546,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>NOVUS RETORNO TOTAL</t>
+          <t>Novus Retorno Total</t>
         </is>
       </c>
       <c r="E23" t="inlineStr"/>
@@ -23584,7 +23584,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>NOVUS LOW VOLATILITY</t>
+          <t>Novus Low Volatility</t>
         </is>
       </c>
       <c r="E24" t="inlineStr"/>
@@ -23622,7 +23622,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>NOVUS PYME FCI ABIERTO PYMES</t>
+          <t>Novus PyME FCI Abierto PyMES</t>
         </is>
       </c>
       <c r="E25" t="inlineStr"/>
@@ -23660,7 +23660,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>NOVUS INCOME DOLARES</t>
+          <t>Novus Income Dolares</t>
         </is>
       </c>
       <c r="E26" t="inlineStr"/>
@@ -23698,7 +23698,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>NOVUS RENTA DÓLAR</t>
+          <t>Novus Renta Dolar</t>
         </is>
       </c>
       <c r="E27" t="inlineStr"/>
@@ -23736,7 +23736,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>NOVUS AHORRO DOLARES</t>
+          <t>Novus Ahorro Dolares</t>
         </is>
       </c>
       <c r="E28" t="inlineStr"/>
@@ -23774,7 +23774,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>NOVUS PERFORMANCE FCI</t>
+          <t>Novus Performance</t>
         </is>
       </c>
       <c r="E29" t="inlineStr"/>
@@ -24316,7 +24316,7 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Novus Dólar MM</t>
+          <t>Novus Dolar MM</t>
         </is>
       </c>
       <c r="E44" t="inlineStr"/>
@@ -24354,7 +24354,7 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Novus Dólar MM</t>
+          <t>Novus Dolar MM</t>
         </is>
       </c>
       <c r="E45" t="inlineStr"/>
@@ -24392,7 +24392,7 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Novus Dólar MM</t>
+          <t>Novus Dolar MM</t>
         </is>
       </c>
       <c r="E46" t="inlineStr"/>
@@ -24430,7 +24430,7 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Novus Dólar MM</t>
+          <t>Novus Dolar MM</t>
         </is>
       </c>
       <c r="E47" t="inlineStr"/>
@@ -24468,7 +24468,7 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Novus Dólar MM</t>
+          <t>Novus Dolar MM</t>
         </is>
       </c>
       <c r="E48" t="inlineStr"/>
@@ -24506,7 +24506,7 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Novus Dólar MM</t>
+          <t>Novus Dolar MM</t>
         </is>
       </c>
       <c r="E49" t="inlineStr"/>
@@ -24544,7 +24544,7 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Novus Dólar MM</t>
+          <t>Novus Dolar MM</t>
         </is>
       </c>
       <c r="E50" t="inlineStr"/>
@@ -24582,7 +24582,7 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Novus Dólar MM</t>
+          <t>Novus Dolar MM</t>
         </is>
       </c>
       <c r="E51" t="inlineStr"/>
@@ -24620,7 +24620,7 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Novus Dólar MM</t>
+          <t>Novus Dolar MM</t>
         </is>
       </c>
       <c r="E52" t="inlineStr"/>
@@ -24658,7 +24658,7 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Novus Dólar MM</t>
+          <t>Novus Dolar MM</t>
         </is>
       </c>
       <c r="E53" t="inlineStr"/>
@@ -24696,7 +24696,7 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Novus Dólar MM</t>
+          <t>Novus Dolar MM</t>
         </is>
       </c>
       <c r="E54" t="inlineStr"/>
@@ -28304,7 +28304,7 @@
       </c>
       <c r="D154" t="inlineStr">
         <is>
-          <t>Novus Gestión II</t>
+          <t>Novus Gestion II</t>
         </is>
       </c>
       <c r="E154" t="inlineStr"/>
@@ -28340,7 +28340,7 @@
       </c>
       <c r="D155" t="inlineStr">
         <is>
-          <t>Novus Gestión II</t>
+          <t>Novus Gestion II</t>
         </is>
       </c>
       <c r="E155" t="inlineStr"/>
@@ -28450,7 +28450,7 @@
       </c>
       <c r="D158" t="inlineStr">
         <is>
-          <t>Novus Dólar MM</t>
+          <t>Novus Dolar MM</t>
         </is>
       </c>
       <c r="E158" t="inlineStr"/>
@@ -28560,7 +28560,7 @@
       </c>
       <c r="D161" t="inlineStr">
         <is>
-          <t>Novus Dólar MM</t>
+          <t>Novus Dolar MM</t>
         </is>
       </c>
       <c r="E161" t="inlineStr"/>

</xml_diff>

<commit_message>
Seguimiento de cuentas · LS · 2026-09-16 18:26
</commit_message>
<xml_diff>
--- a/data/seguimiento_cuentas.xlsx
+++ b/data/seguimiento_cuentas.xlsx
@@ -1700,7 +1700,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Alynk S.A.</t>
+          <t>Alynk</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -1738,7 +1738,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Alynk S.A.</t>
+          <t>Alynk</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -1776,7 +1776,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Alynk S.A.</t>
+          <t>Alynk</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -1814,7 +1814,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Alynk S.A.</t>
+          <t>Alynk</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -1852,7 +1852,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Alynk S.A.</t>
+          <t>Alynk</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -1890,7 +1890,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Alynk S.A.</t>
+          <t>Alynk</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -1928,7 +1928,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Alynk S.A.</t>
+          <t>Alynk</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -1966,7 +1966,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Alynk S.A.</t>
+          <t>Alynk</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -2046,7 +2046,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Alynk S.A.</t>
+          <t>Alynk</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -2084,7 +2084,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Alynk S.A.</t>
+          <t>Alynk</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -2122,7 +2122,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Alynk S.A.</t>
+          <t>Alynk</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -2160,7 +2160,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Alynk S.A.</t>
+          <t>Alynk</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -2198,7 +2198,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Alynk S.A.</t>
+          <t>Alynk</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -2270,7 +2270,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Alynk S.A.</t>
+          <t>Alynk</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -2308,7 +2308,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Alynk S.A.</t>
+          <t>Alynk</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -2346,7 +2346,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Alynk S.A.</t>
+          <t>Alynk</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -2384,7 +2384,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Alynk S.A.</t>
+          <t>Alynk</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -2422,7 +2422,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Alynk S.A.</t>
+          <t>Alynk</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -2536,7 +2536,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Santander Valores</t>
+          <t>Banco Santander</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -3606,7 +3606,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>Option</t>
+          <t>Option Securities S.A.</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
@@ -5220,7 +5220,7 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>Bapro</t>
+          <t>BAPRO</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
@@ -5280,7 +5280,7 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>Cohen S.A.</t>
+          <t>Cohen</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
@@ -5318,7 +5318,7 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>Cohen S.A.</t>
+          <t>Cohen</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
@@ -5356,7 +5356,7 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>Cohen S.A.</t>
+          <t>Cohen</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
@@ -6134,7 +6134,7 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>Comafi</t>
+          <t>Banco Comafi</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
@@ -6164,7 +6164,7 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>Fynsa</t>
+          <t>FYNSA</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
@@ -6346,7 +6346,7 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>Galicia</t>
+          <t>Banco Galicia</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
@@ -6570,7 +6570,7 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>Grit</t>
+          <t>Grit Capital</t>
         </is>
       </c>
       <c r="C165" t="inlineStr">
@@ -7208,7 +7208,7 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>IEB Fondos</t>
+          <t>IEB FONDOS</t>
         </is>
       </c>
       <c r="C182" t="inlineStr">
@@ -7314,7 +7314,7 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>Fynsa</t>
+          <t>FYNSA</t>
         </is>
       </c>
       <c r="C185" t="inlineStr">
@@ -7348,7 +7348,7 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>Option Securities</t>
+          <t>Option Securities S.A.</t>
         </is>
       </c>
       <c r="C186" t="inlineStr">
@@ -7382,7 +7382,7 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>Option Securities</t>
+          <t>Option Securities S.A.</t>
         </is>
       </c>
       <c r="C187" t="inlineStr">
@@ -7518,7 +7518,7 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>Puente Hnos</t>
+          <t>Puente Hnos.</t>
         </is>
       </c>
       <c r="C191" t="inlineStr">
@@ -7856,7 +7856,7 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>Industrial</t>
+          <t>Banco Industrial S.A.</t>
         </is>
       </c>
       <c r="C200" t="inlineStr">
@@ -8266,7 +8266,7 @@
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>Latin</t>
+          <t>Latin Securities</t>
         </is>
       </c>
       <c r="C211" t="inlineStr">
@@ -8422,7 +8422,7 @@
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>Macro</t>
+          <t>Banco Macro</t>
         </is>
       </c>
       <c r="C215" t="inlineStr">
@@ -8452,7 +8452,7 @@
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>Macro Securities</t>
+          <t>Banco Macro</t>
         </is>
       </c>
       <c r="C216" t="inlineStr">
@@ -8520,7 +8520,7 @@
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>Mariva</t>
+          <t>Banco Mariva</t>
         </is>
       </c>
       <c r="C218" t="inlineStr">
@@ -8580,7 +8580,7 @@
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>Option</t>
+          <t>Option Securities S.A.</t>
         </is>
       </c>
       <c r="C220" t="inlineStr">
@@ -8644,7 +8644,7 @@
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>Puente</t>
+          <t>Puente Hnos.</t>
         </is>
       </c>
       <c r="C222" t="inlineStr">
@@ -8818,7 +8818,7 @@
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>Supervielle</t>
+          <t>Banco Supervielle</t>
         </is>
       </c>
       <c r="C227" t="inlineStr">
@@ -10628,7 +10628,7 @@
       </c>
       <c r="B274" t="inlineStr">
         <is>
-          <t>Puente Hnos</t>
+          <t>Puente Hnos.</t>
         </is>
       </c>
       <c r="C274" t="inlineStr">
@@ -13180,7 +13180,7 @@
       </c>
       <c r="B342" t="inlineStr">
         <is>
-          <t>Option</t>
+          <t>Option Securities S.A.</t>
         </is>
       </c>
       <c r="C342" t="inlineStr">
@@ -13718,7 +13718,7 @@
       </c>
       <c r="B357" t="inlineStr">
         <is>
-          <t>Santander Valores</t>
+          <t>Banco Santander</t>
         </is>
       </c>
       <c r="C357" t="inlineStr">
@@ -13756,7 +13756,7 @@
       </c>
       <c r="B358" t="inlineStr">
         <is>
-          <t>Santander Valores</t>
+          <t>Banco Santander</t>
         </is>
       </c>
       <c r="C358" t="inlineStr">
@@ -13794,7 +13794,7 @@
       </c>
       <c r="B359" t="inlineStr">
         <is>
-          <t>Santander Valores</t>
+          <t>Banco Santander</t>
         </is>
       </c>
       <c r="C359" t="inlineStr">
@@ -13832,7 +13832,7 @@
       </c>
       <c r="B360" t="inlineStr">
         <is>
-          <t>Santander Valores</t>
+          <t>Banco Santander</t>
         </is>
       </c>
       <c r="C360" t="inlineStr">
@@ -13870,7 +13870,7 @@
       </c>
       <c r="B361" t="inlineStr">
         <is>
-          <t>Santander Valores</t>
+          <t>Banco Santander</t>
         </is>
       </c>
       <c r="C361" t="inlineStr">
@@ -13942,7 +13942,7 @@
       </c>
       <c r="B363" t="inlineStr">
         <is>
-          <t>Santander Valores</t>
+          <t>Banco Santander</t>
         </is>
       </c>
       <c r="C363" t="inlineStr">
@@ -13980,7 +13980,7 @@
       </c>
       <c r="B364" t="inlineStr">
         <is>
-          <t>Santander Valores</t>
+          <t>Banco Santander</t>
         </is>
       </c>
       <c r="C364" t="inlineStr">
@@ -14018,7 +14018,7 @@
       </c>
       <c r="B365" t="inlineStr">
         <is>
-          <t>Santander Valores</t>
+          <t>Banco Santander</t>
         </is>
       </c>
       <c r="C365" t="inlineStr">
@@ -14056,7 +14056,7 @@
       </c>
       <c r="B366" t="inlineStr">
         <is>
-          <t>Santander Valores</t>
+          <t>Banco Santander</t>
         </is>
       </c>
       <c r="C366" t="inlineStr">
@@ -14094,7 +14094,7 @@
       </c>
       <c r="B367" t="inlineStr">
         <is>
-          <t>Santander Valores</t>
+          <t>Banco Santander</t>
         </is>
       </c>
       <c r="C367" t="inlineStr">
@@ -14132,7 +14132,7 @@
       </c>
       <c r="B368" t="inlineStr">
         <is>
-          <t>Santander Valores</t>
+          <t>Banco Santander</t>
         </is>
       </c>
       <c r="C368" t="inlineStr">
@@ -14170,7 +14170,7 @@
       </c>
       <c r="B369" t="inlineStr">
         <is>
-          <t>Santander Valores</t>
+          <t>Banco Santander</t>
         </is>
       </c>
       <c r="C369" t="inlineStr">
@@ -14208,7 +14208,7 @@
       </c>
       <c r="B370" t="inlineStr">
         <is>
-          <t>Santander Valores</t>
+          <t>Banco Santander</t>
         </is>
       </c>
       <c r="C370" t="inlineStr">
@@ -14246,7 +14246,7 @@
       </c>
       <c r="B371" t="inlineStr">
         <is>
-          <t>Santander Valores</t>
+          <t>Banco Santander</t>
         </is>
       </c>
       <c r="C371" t="inlineStr">
@@ -14322,7 +14322,7 @@
       </c>
       <c r="B373" t="inlineStr">
         <is>
-          <t>Santander Valores</t>
+          <t>Banco Santander</t>
         </is>
       </c>
       <c r="C373" t="inlineStr">
@@ -14360,7 +14360,7 @@
       </c>
       <c r="B374" t="inlineStr">
         <is>
-          <t>Santander Valores</t>
+          <t>Banco Santander</t>
         </is>
       </c>
       <c r="C374" t="inlineStr">
@@ -14398,7 +14398,7 @@
       </c>
       <c r="B375" t="inlineStr">
         <is>
-          <t>Santander Valores</t>
+          <t>Banco Santander</t>
         </is>
       </c>
       <c r="C375" t="inlineStr">
@@ -14436,7 +14436,7 @@
       </c>
       <c r="B376" t="inlineStr">
         <is>
-          <t>Santander Valores</t>
+          <t>Banco Santander</t>
         </is>
       </c>
       <c r="C376" t="inlineStr">
@@ -14474,7 +14474,7 @@
       </c>
       <c r="B377" t="inlineStr">
         <is>
-          <t>Santander Valores</t>
+          <t>Banco Santander</t>
         </is>
       </c>
       <c r="C377" t="inlineStr">
@@ -14512,7 +14512,7 @@
       </c>
       <c r="B378" t="inlineStr">
         <is>
-          <t>Santander Valores</t>
+          <t>Banco Santander</t>
         </is>
       </c>
       <c r="C378" t="inlineStr">
@@ -14550,7 +14550,7 @@
       </c>
       <c r="B379" t="inlineStr">
         <is>
-          <t>Alynk S.A.</t>
+          <t>Alynk</t>
         </is>
       </c>
       <c r="C379" t="inlineStr">
@@ -15444,7 +15444,7 @@
       </c>
       <c r="B404" t="inlineStr">
         <is>
-          <t>Santander Valores</t>
+          <t>Banco Santander</t>
         </is>
       </c>
       <c r="C404" t="inlineStr">
@@ -17408,7 +17408,7 @@
       </c>
       <c r="B458" t="inlineStr">
         <is>
-          <t>Alynk S.A.</t>
+          <t>Alynk</t>
         </is>
       </c>
       <c r="C458" t="inlineStr">
@@ -19570,7 +19570,7 @@
       </c>
       <c r="B519" t="inlineStr">
         <is>
-          <t>Santander Valores</t>
+          <t>Banco Santander</t>
         </is>
       </c>
       <c r="C519" t="inlineStr">
@@ -19986,7 +19986,7 @@
       </c>
       <c r="B531" t="inlineStr">
         <is>
-          <t>Option</t>
+          <t>Option Securities S.A.</t>
         </is>
       </c>
       <c r="C531" t="inlineStr">
@@ -20020,7 +20020,7 @@
       </c>
       <c r="B532" t="inlineStr">
         <is>
-          <t>Option</t>
+          <t>Option Securities S.A.</t>
         </is>
       </c>
       <c r="C532" t="inlineStr">
@@ -21098,7 +21098,7 @@
       </c>
       <c r="B563" t="inlineStr">
         <is>
-          <t>PUENTE</t>
+          <t>Puente Hnos.</t>
         </is>
       </c>
       <c r="C563" t="inlineStr">
@@ -21136,7 +21136,7 @@
       </c>
       <c r="B564" t="inlineStr">
         <is>
-          <t>Mariva</t>
+          <t>Banco Mariva</t>
         </is>
       </c>
       <c r="C564" t="inlineStr">
@@ -22538,7 +22538,7 @@
       </c>
       <c r="B601" t="inlineStr">
         <is>
-          <t>Allaria Alyc</t>
+          <t>Allaria</t>
         </is>
       </c>
       <c r="C601" t="inlineStr">
@@ -22819,7 +22819,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Banco Industrial</t>
+          <t>Banco Industrial S.A.</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -24349,7 +24349,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Banco Nacion</t>
+          <t>Banco Nación</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -24387,7 +24387,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Supervielle</t>
+          <t>Banco Supervielle</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -24501,7 +24501,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Banco GaLICIA</t>
+          <t>Banco Galicia</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -24615,7 +24615,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Macro</t>
+          <t>Banco Macro</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -24653,7 +24653,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Valores</t>
+          <t>Banco de Valores</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -25347,7 +25347,7 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Banco Nacion</t>
+          <t>Banco Nación</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
@@ -27795,7 +27795,7 @@
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>Banco Comafi S.A.</t>
+          <t>Banco Comafi</t>
         </is>
       </c>
       <c r="D140" t="inlineStr">
@@ -27903,7 +27903,7 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>Banco Mariva S.A.</t>
+          <t>Banco Mariva</t>
         </is>
       </c>
       <c r="D143" t="inlineStr">
@@ -27939,7 +27939,7 @@
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>Banco Supervielle S.A.</t>
+          <t>Banco Supervielle</t>
         </is>
       </c>
       <c r="D144" t="inlineStr">
@@ -27975,7 +27975,7 @@
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>Banco Comafi S.A.</t>
+          <t>Banco Comafi</t>
         </is>
       </c>
       <c r="D145" t="inlineStr">
@@ -28083,7 +28083,7 @@
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>Banco Mariva S.A.</t>
+          <t>Banco Mariva</t>
         </is>
       </c>
       <c r="D148" t="inlineStr">
@@ -28119,7 +28119,7 @@
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>Banco Supervielle S.A.</t>
+          <t>Banco Supervielle</t>
         </is>
       </c>
       <c r="D149" t="inlineStr">
@@ -28155,7 +28155,7 @@
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>Banco Comafi S.A.</t>
+          <t>Banco Comafi</t>
         </is>
       </c>
       <c r="D150" t="inlineStr">
@@ -28335,7 +28335,7 @@
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>Banco Supervielle S.A.</t>
+          <t>Banco Supervielle</t>
         </is>
       </c>
       <c r="D155" t="inlineStr">
@@ -28407,7 +28407,7 @@
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>Banco Supervielle S.A.</t>
+          <t>Banco Supervielle</t>
         </is>
       </c>
       <c r="D157" t="inlineStr">

</xml_diff>

<commit_message>
Seguimiento de cuentas · LS · 2026-09-16 18:29
</commit_message>
<xml_diff>
--- a/data/seguimiento_cuentas.xlsx
+++ b/data/seguimiento_cuentas.xlsx
@@ -22677,7 +22677,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J166"/>
+  <dimension ref="A1:J165"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -28618,7 +28618,7 @@
     </row>
     <row r="163">
       <c r="A163" s="1" t="n">
-        <v>46269</v>
+        <v>46280</v>
       </c>
       <c r="B163" t="inlineStr">
         <is>
@@ -28632,19 +28632,19 @@
       </c>
       <c r="D163" t="inlineStr">
         <is>
-          <t>Novus Renta Variable</t>
+          <t>Novus PyME FCI Abierto PyMES</t>
         </is>
       </c>
       <c r="E163" t="inlineStr"/>
       <c r="F163" t="inlineStr">
         <is>
-          <t>En proceso</t>
+          <t>Abierta</t>
         </is>
       </c>
       <c r="G163" t="inlineStr"/>
       <c r="H163" t="inlineStr">
         <is>
-          <t>1. Inicio / Solicitud</t>
+          <t>4. Exención ARCA</t>
         </is>
       </c>
       <c r="I163" t="inlineStr"/>
@@ -28666,19 +28666,19 @@
       </c>
       <c r="D164" t="inlineStr">
         <is>
-          <t>Novus PyME FCI Abierto PyMES</t>
+          <t>Novus Renta Variable</t>
         </is>
       </c>
       <c r="E164" t="inlineStr"/>
       <c r="F164" t="inlineStr">
         <is>
-          <t>Abierta</t>
+          <t>En proceso</t>
         </is>
       </c>
       <c r="G164" t="inlineStr"/>
       <c r="H164" t="inlineStr">
         <is>
-          <t>4. Exención ARCA</t>
+          <t>3. Doc SD</t>
         </is>
       </c>
       <c r="I164" t="inlineStr"/>
@@ -28686,7 +28686,7 @@
     </row>
     <row r="165">
       <c r="A165" s="1" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="B165" t="inlineStr">
         <is>
@@ -28700,57 +28700,23 @@
       </c>
       <c r="D165" t="inlineStr">
         <is>
-          <t>Novus Renta Variable</t>
+          <t>Novus Renta Capital</t>
         </is>
       </c>
       <c r="E165" t="inlineStr"/>
       <c r="F165" t="inlineStr">
         <is>
-          <t>En proceso</t>
+          <t>Abierta</t>
         </is>
       </c>
       <c r="G165" t="inlineStr"/>
       <c r="H165" t="inlineStr">
         <is>
-          <t>3. Doc SD</t>
+          <t>5. Habilitada para operar</t>
         </is>
       </c>
       <c r="I165" t="inlineStr"/>
       <c r="J165" t="inlineStr"/>
-    </row>
-    <row r="166">
-      <c r="A166" s="1" t="n">
-        <v>46281</v>
-      </c>
-      <c r="B166" t="inlineStr">
-        <is>
-          <t>Remunerada</t>
-        </is>
-      </c>
-      <c r="C166" t="inlineStr">
-        <is>
-          <t>Banco Supervielle</t>
-        </is>
-      </c>
-      <c r="D166" t="inlineStr">
-        <is>
-          <t>Novus Renta Capital</t>
-        </is>
-      </c>
-      <c r="E166" t="inlineStr"/>
-      <c r="F166" t="inlineStr">
-        <is>
-          <t>Abierta</t>
-        </is>
-      </c>
-      <c r="G166" t="inlineStr"/>
-      <c r="H166" t="inlineStr">
-        <is>
-          <t>5. Habilitada para operar</t>
-        </is>
-      </c>
-      <c r="I166" t="inlineStr"/>
-      <c r="J166" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>